<commit_message>
Update course offerings and course plans in various subjects
- Added new courses to the Philosophy MOC and updated the count of active courses.
- Updated the number of inactive course plans in the Philosophy MOC.
- Modified the number of courses in the ISLL MOC for Arabic, English, French, Japanese, Chinese, and Swedish.
- Added new courses to the English MOC and adjusted the count of active and inactive courses.
- Updated course plans for various subjects, including English and French, reflecting changes in course availability.
- Adjusted the number of problematic course plans and their respective download links in the analysis documents.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E204"/>
+  <dimension ref="A1:E203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1481,12 +1481,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>`europeiskspråkiga` (sv)</t>
+          <t>`poitical` (en)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -1498,7 +1498,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>AHI272</t>
+          <t>AHI29Q</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1513,12 +1513,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>`poitical` (en)</t>
+          <t>`consultaion` (en)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AHI272</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AHI29Q</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>`consultaion` (en)</t>
+          <t>`situatin` (en)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>AHI29Q</t>
+          <t>AS2005</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1567,19 +1567,19 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>`situatin` (en)</t>
+          <t>`takenup` (en)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AHI29Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS2005</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>AS2005</t>
+          <t>AS3017</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1589,24 +1589,24 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>`takenup` (en)</t>
+          <t>`literära` (sv)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS2005</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3017</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>AS3017</t>
+          <t>AS3020</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1616,24 +1616,24 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>`literära` (sv)</t>
+          <t>`outlineof` (en)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3020</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>AS3020</t>
+          <t>AS3022</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1648,19 +1648,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>`outlineof` (en)</t>
+          <t>`teh` (en)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3022</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>AS3022</t>
+          <t>GHI29Y</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1670,24 +1670,24 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>`teh` (en)</t>
+          <t>`innhållet` (sv)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI29Y</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>GHI29Y</t>
+          <t>GHI33T</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1702,19 +1702,19 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>`innhållet` (sv)</t>
+          <t>`problemförmuleringsförmåga` (sv)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI29Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI33T</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>GHI33T</t>
+          <t>GHI33V</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1729,12 +1729,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>`problemförmuleringsförmåga` (sv)</t>
+          <t>`delkurseninnehåller` (sv)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI33T</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI33V</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>`delkurseninnehåller` (sv)</t>
+          <t>`godkäng` (sv)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -1768,7 +1768,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>GHI33V</t>
+          <t>GHI35A</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1783,12 +1783,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>`godkäng` (sv)</t>
+          <t>`analyseratmänniskors` (sv)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI33V</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI35A</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>`analyseratmänniskors` (sv)</t>
+          <t>`medförintelsen` (sv)</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>`medförintelsen` (sv)</t>
+          <t>`människorsagerande` (sv)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -1849,7 +1849,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>GHI35A</t>
+          <t>GHI362</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1864,19 +1864,19 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>`människorsagerande` (sv)</t>
+          <t>`självstänigt` (sv)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI35A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI362</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>GHI362</t>
+          <t>HI1008</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1886,24 +1886,24 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>`självstänigt` (sv)</t>
+          <t>`criterions` (en)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GHI362</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI1008</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>HI1008</t>
+          <t>HI2011</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1913,24 +1913,24 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>`criterions` (en)</t>
+          <t>`historiedidaktikområdet` (sv)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI1008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI2011</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>HI2011</t>
+          <t>HI2012</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1945,19 +1945,19 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>`historiedidaktikområdet` (sv)</t>
+          <t>`sjävvalt` (sv)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI2011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI2012</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>HI2012</t>
+          <t>HI2016</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1977,14 +1977,14 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI2012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI2016</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>HI2016</t>
+          <t>HI3019</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1999,39 +1999,39 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>`sjävvalt` (sv)</t>
+          <t>`självständg` (sv)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI2016</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI3019</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>HI3019</t>
+          <t>AKG27R</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>HIA</t>
+          <t>KGA</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>`självständg` (sv)</t>
+          <t>`compulsotry` (en)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=HI3019</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AKG27R</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2053,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>`compulsotry` (en)</t>
+          <t>`curent` (en)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2080,7 +2080,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>`curent` (en)</t>
+          <t>`theoretica` (en)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -2092,7 +2092,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>AKG27R</t>
+          <t>GKG3AT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2102,17 +2102,17 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>`theoretica` (en)</t>
+          <t>`tilllämpas` (sv)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AKG27R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKG3AT</t>
         </is>
       </c>
     </row>
@@ -2129,12 +2129,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>`tilllämpas` (sv)</t>
+          <t>`writtten` (en)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
@@ -2146,7 +2146,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GKG3AT</t>
+          <t>KG1024</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2156,17 +2156,17 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>`writtten` (en)</t>
+          <t>`beräklningstung` (sv)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GKG3AT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG1024</t>
         </is>
       </c>
     </row>
@@ -2183,12 +2183,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>`beräklningstung` (sv)</t>
+          <t>`quantitativ` (en)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -2200,7 +2200,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>KG1024</t>
+          <t>KG1025</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2215,12 +2215,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>`quantitativ` (en)</t>
+          <t>`evolvement` (en)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG1025</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>`evolvement` (en)</t>
+          <t>`thise` (en)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -2254,7 +2254,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>KG1025</t>
+          <t>KG2001</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2269,12 +2269,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>`thise` (en)</t>
+          <t>`obser` (en)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG1025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG2001</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>`obser` (en)</t>
+          <t>`perspetives` (en)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>`perspetives` (en)</t>
+          <t>`standarized` (en)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>`standarized` (en)</t>
+          <t>`vations` (en)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -2362,7 +2362,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>KG2001</t>
+          <t>KG2005</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>`vations` (en)</t>
+          <t>`qualititative` (en)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG2001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG2005</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>KG2005</t>
+          <t>KG3010</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>`qualititative` (en)</t>
+          <t>`recognises` (en)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG2005</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3010</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>KG3010</t>
+          <t>KG3011</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2426,17 +2426,17 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>`recognises` (en)</t>
+          <t>`kartöverlägg` (sv)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3010</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3011</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>`kartöverlägg` (sv)</t>
+          <t>`skalnivå` (sv)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
@@ -2470,7 +2470,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>KG3011</t>
+          <t>KG3014</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2480,24 +2480,24 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>`skalnivå` (sv)</t>
+          <t>`eaxaminer` (en)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3014</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>KG3014</t>
+          <t>KG3015</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2517,14 +2517,14 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3015</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>KG3015</t>
+          <t>KG3016</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2534,29 +2534,29 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>`eaxaminer` (en)</t>
+          <t>`gällade` (sv)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3016</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>KG3016</t>
+          <t>GLP236</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>KGA</t>
+          <t>LPU</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2566,19 +2566,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>`gällade` (sv)</t>
+          <t>`framträdandeform` (sv)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=KG3016</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP236</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GLP236</t>
+          <t>GLP29R</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2593,19 +2593,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>`framträdandeform` (sv)</t>
+          <t>`flerspårsmaterial` (sv)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP236</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP29R</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GLP29R</t>
+          <t>GLP2JZ</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2625,14 +2625,14 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP29R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2JZ</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GLP2JZ</t>
+          <t>GLP359</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2642,24 +2642,24 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>`flerspårsmaterial` (sv)</t>
+          <t>`djing` (en)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP2JZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP359</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GLP359</t>
+          <t>GLP3AH</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2674,19 +2674,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>`djing` (en)</t>
+          <t>`excercises` (en)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP359</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP3AH</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GLP3AH</t>
+          <t>LP1032</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2696,17 +2696,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>`excercises` (en)</t>
+          <t>`fördjupningskod` (sv)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GLP3AH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP1032</t>
         </is>
       </c>
     </row>
@@ -2723,12 +2723,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>`fördjupningskod` (sv)</t>
+          <t>`scholary` (en)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>`scholary` (en)</t>
+          <t>`sumarise` (en)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -2767,7 +2767,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>LP1032</t>
+          <t>LP1071</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2777,17 +2777,17 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>`sumarise` (en)</t>
+          <t>`erätter` (sv)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP1032</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP1071</t>
         </is>
       </c>
     </row>
@@ -2804,12 +2804,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>`erätter` (sv)</t>
+          <t>`evaulates` (en)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -2821,7 +2821,7 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>LP1071</t>
+          <t>LP2012</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2836,19 +2836,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>`evaulates` (en)</t>
+          <t>`intiate` (en)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP1071</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP2012</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>LP2012</t>
+          <t>LP2013</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>`intiate` (en)</t>
+          <t>`learnings` (en)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP2012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP2013</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>`learnings` (en)</t>
+          <t>`litterature` (en)</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -2902,39 +2902,39 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>LP2013</t>
+          <t>GMN3EA</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>LPU</t>
+          <t>MPR</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>`litterature` (en)</t>
+          <t>`användar` (sv)</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=LP2013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3EA</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>GMN3EA</t>
+          <t>NA1024</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MPR</t>
+          <t>NAA</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2944,12 +2944,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>`användar` (sv)</t>
+          <t>`efterfråge` (sv)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMN3EA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1024</t>
         </is>
       </c>
     </row>
@@ -2966,12 +2966,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>`efterfråge` (sv)</t>
+          <t>`distancelectures` (en)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -2983,7 +2983,7 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>NA1024</t>
+          <t>NA1026</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2993,24 +2993,24 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>`distancelectures` (en)</t>
+          <t>`studieförb` (sv)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>NA1026</t>
+          <t>NA1027</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -3025,19 +3025,19 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>`studieförb` (sv)</t>
+          <t>`förläsningar` (sv)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1026</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1027</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>NA1027</t>
+          <t>NA1028</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -3052,19 +3052,19 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>`förläsningar` (sv)</t>
+          <t>`efterfråge` (sv)</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1028</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>NA1028</t>
+          <t>NA1029</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -3074,24 +3074,24 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>`efterfråge` (sv)</t>
+          <t>`differentiat` (en)</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1028</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1029</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>NA1029</t>
+          <t>NA1030</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -3106,19 +3106,19 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>`differentiat` (en)</t>
+          <t>`excercises` (en)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1029</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1030</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>NA1030</t>
+          <t>NA1032</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3133,19 +3133,19 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>`excercises` (en)</t>
+          <t>`descirbe` (en)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1030</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1032</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>NA1032</t>
+          <t>NA1035</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3155,24 +3155,24 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>`descirbe` (en)</t>
+          <t>`efterfråge` (sv)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1032</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1035</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>NA1035</t>
+          <t>NA1036</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3182,17 +3182,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>`efterfråge` (sv)</t>
+          <t>`longterm` (en)</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1035</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1036</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3214,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>`longterm` (en)</t>
+          <t>`shortterm` (en)</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
@@ -3226,7 +3226,7 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>NA1036</t>
+          <t>NA1039</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3241,19 +3241,19 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>`shortterm` (en)</t>
+          <t>`assingments` (en)</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1036</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1039</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>NA1039</t>
+          <t>NA2008</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3263,17 +3263,17 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>`assingments` (en)</t>
+          <t>`kalandermånader` (sv)</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA1039</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA2008</t>
         </is>
       </c>
     </row>
@@ -3290,12 +3290,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>`kalandermånader` (sv)</t>
+          <t>`calender` (en)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>`calender` (en)</t>
+          <t>`oppobet` (en)</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>`oppobet` (en)</t>
+          <t>`opposnent` (en)</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
@@ -3361,7 +3361,7 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>NA2008</t>
+          <t>NA2009</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3376,19 +3376,19 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>`opposnent` (en)</t>
+          <t>`resultas` (en)</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA2008</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA2009</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>NA2009</t>
+          <t>NA3001</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3398,24 +3398,24 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>`resultas` (en)</t>
+          <t>`länderjämförelser` (sv)</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA2009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3001</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>NA3001</t>
+          <t>NA3010</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3430,19 +3430,19 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>`länderjämförelser` (sv)</t>
+          <t>`kalandermånader` (sv)</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3010</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>NA3010</t>
+          <t>NA3011</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3452,51 +3452,51 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>`kalandermånader` (sv)</t>
+          <t>`tobbit` (en)</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3010</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3011</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>NA3011</t>
+          <t>GPE3AJ</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>NAA</t>
+          <t>PEA</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>`tobbit` (en)</t>
+          <t>`kollegialtlärande` (sv)</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=NA3011</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPE3AJ</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>GPE3AJ</t>
+          <t>PE1020</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3506,24 +3506,24 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>`kollegialtlärande` (sv)</t>
+          <t>`gryndsyn` (en)</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPE3AJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1020</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>PE1020</t>
+          <t>PE1023</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3533,17 +3533,17 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>`gryndsyn` (en)</t>
+          <t>`lärarlagsarbete` (sv)</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1020</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1023</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3565,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>`lärarlagsarbete` (sv)</t>
+          <t>`rättsäkerhet` (sv)</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
@@ -3577,7 +3577,7 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>PE1023</t>
+          <t>PE1054</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3592,19 +3592,19 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>`rättsäkerhet` (sv)</t>
+          <t>`lärstrategier` (sv)</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1023</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1054</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>PE1054</t>
+          <t>PE1064</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3619,19 +3619,19 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>`lärstrategier` (sv)</t>
+          <t>`rättsäkerhetsproblematiken` (sv)</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1054</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1064</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>PE1064</t>
+          <t>PE1067</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3641,24 +3641,24 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>`rättsäkerhetsproblematiken` (sv)</t>
+          <t>`att` — ….m. 2014-01-24.  ## Lärandemål  Kursens övergripande mål är att att den studerande förstår hur man kan styra sina informationsf…</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1067</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>PE1067</t>
+          <t>PE1068</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3668,24 +3668,24 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>`att` — ….m. 2014-01-24.  ## Lärandemål  Kursens övergripande mål är att att den studerande förstår hur man kan styra sina informationsf…</t>
+          <t>`känndom` (sv)</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1067</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1068</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>PE1068</t>
+          <t>PE2005</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3695,24 +3695,24 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>`känndom` (sv)</t>
+          <t>`gryndsyn` (en)</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE2005</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>PE2005</t>
+          <t>PE3004</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3722,17 +3722,17 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>`gryndsyn` (en)</t>
+          <t>`lärarlagsarbete` (sv)</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE2005</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE3004</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>`lärarlagsarbete` (sv)</t>
+          <t>`rättsäkerhet` (sv)</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
@@ -3766,34 +3766,34 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>PE3004</t>
+          <t>GPA2FW</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>PEA</t>
+          <t>PEE</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>`rättsäkerhet` (sv)</t>
+          <t>`managemet` (en)</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=PE3004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2FW</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>GPA2FW</t>
+          <t>GPA2R6</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3803,29 +3803,29 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>`managemet` (en)</t>
+          <t>`tillvägagångsätt` (sv)</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2FW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2R6</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>GPA2R6</t>
+          <t>APG24E</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>PEE</t>
+          <t>PGA</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3835,12 +3835,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>`tillvägagångsätt` (sv)</t>
+          <t>`inlämingsuppgifter` (sv)</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPA2R6</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG24E</t>
         </is>
       </c>
     </row>
@@ -3857,12 +3857,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>`inlämingsuppgifter` (sv)</t>
+          <t>`credtis` (en)</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
@@ -3874,7 +3874,7 @@
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>APG24E</t>
+          <t>APG25N</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3884,24 +3884,24 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>`credtis` (en)</t>
+          <t>`tillvägagångsätt` (sv)</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG24E</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG25N</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>APG25N</t>
+          <t>APG276</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3911,24 +3911,24 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>`tillvägagångsätt` (sv)</t>
+          <t>`credtis` (en)</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG25N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG276</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>APG276</t>
+          <t>APG2AA</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3938,24 +3938,24 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>`credtis` (en)</t>
+          <t>`lärarskicklighetetens` (sv)</t>
         </is>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG276</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2AA</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>APG2AA</t>
+          <t>APG2AC</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3965,17 +3965,17 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>`lärarskicklighetetens` (sv)</t>
+          <t>`aanalyze` (en)</t>
         </is>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2AA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2AC</t>
         </is>
       </c>
     </row>
@@ -3997,7 +3997,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>`aanalyze` (en)</t>
+          <t>`nalyze` (en)</t>
         </is>
       </c>
       <c r="E132" s="2" t="inlineStr">
@@ -4009,7 +4009,7 @@
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>APG2AC</t>
+          <t>APG2CD</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -4019,24 +4019,24 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>`nalyze` (en)</t>
+          <t>`lärarprofessionsspecifika` (sv)</t>
         </is>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2AC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2CD</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>APG2CD</t>
+          <t>APG2CM</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -4051,19 +4051,19 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>`lärarprofessionsspecifika` (sv)</t>
+          <t>`undervisningensmål` (sv)</t>
         </is>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2CD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2CM</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>APG2CM</t>
+          <t>GPG22K</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -4073,24 +4073,24 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>`undervisningensmål` (sv)</t>
+          <t>`conciderations` (en)</t>
         </is>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=APG2CM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG22K</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>GPG22K</t>
+          <t>GPG2SC</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -4100,17 +4100,17 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>`conciderations` (en)</t>
+          <t>`samhällorienterande` (sv)</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG22K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG2SC</t>
         </is>
       </c>
     </row>
@@ -4127,12 +4127,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>`samhällorienterande` (sv)</t>
+          <t>`sociaty` (en)</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>`sociaty` (en)</t>
+          <t>`understandingn` (en)</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
@@ -4171,7 +4171,7 @@
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>GPG2SC</t>
+          <t>GPG328</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -4181,24 +4181,24 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>`understandingn` (en)</t>
+          <t>`andraämne` (sv)</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG2SC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG328</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>GPG328</t>
+          <t>GPG329</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -4218,14 +4218,14 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG328</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG329</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>GPG329</t>
+          <t>GPG3AD</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -4235,24 +4235,24 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>`andraämne` (sv)</t>
+          <t>`as` — …ment on the way to the subject teaching profession, as well as as support for being able to make conscious didactic choices d…</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG329</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3AD</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>GPG3AD</t>
+          <t>GPG3CG</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -4262,24 +4262,24 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>`as` — …ment on the way to the subject teaching profession, as well as as support for being able to make conscious didactic choices d…</t>
+          <t>`perspecitves` (en)</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3AD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CG</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>GPG3CG</t>
+          <t>GPG3CK</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -4289,24 +4289,24 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>`perspecitves` (en)</t>
+          <t>`inlämninguppgift` (sv)</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CK</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>GPG3CK</t>
+          <t>GPG3CL</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -4321,12 +4321,12 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>`inlämninguppgift` (sv)</t>
+          <t>`samhällorienterande` (sv)</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CL</t>
         </is>
       </c>
     </row>
@@ -4343,12 +4343,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>`samhällorienterande` (sv)</t>
+          <t>`sociaty` (en)</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
@@ -4360,12 +4360,12 @@
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>GPG3CL</t>
+          <t>ARK27Q</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>PGA</t>
+          <t>RKA</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -4375,19 +4375,19 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>`sociaty` (en)</t>
+          <t>`tha` (en)</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG3CL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK27Q</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>ARK27Q</t>
+          <t>ARK29K</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -4402,19 +4402,19 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>`tha` (en)</t>
+          <t>`cpecialisation` (en)</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK27Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29K</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>ARK29K</t>
+          <t>ARK29L</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4424,24 +4424,24 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>`cpecialisation` (en)</t>
+          <t>`markonivå` (sv)</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29L</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>ARK29L</t>
+          <t>GRK366</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4451,24 +4451,24 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>`markonivå` (sv)</t>
+          <t>`enivronments` (en)</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ARK29L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK366</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>GRK366</t>
+          <t>GRK3B4</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4478,29 +4478,29 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>`enivronments` (en)</t>
+          <t>`ämesteoretiska` (sv)</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK366</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK3B4</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>GRK3B4</t>
+          <t>GRV266</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>RKA</t>
+          <t>RVA</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -4510,19 +4510,19 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>`ämesteoretiska` (sv)</t>
+          <t>`mervärdskatt` (sv)</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRK3B4</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRV266</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>GRV266</t>
+          <t>GRV2MK</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4537,19 +4537,19 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>`mervärdskatt` (sv)</t>
+          <t>`innhåller` (sv)</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRV266</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRV2MK</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>GRV2MK</t>
+          <t>RV1001</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4564,19 +4564,19 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>`innhåller` (sv)</t>
+          <t>`glavå` (sv)</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GRV2MK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1001</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>RV1001</t>
+          <t>RV1003</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4591,19 +4591,19 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>`glavå` (sv)</t>
+          <t>`mervärdskatt` (sv)</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1003</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>RV1003</t>
+          <t>RV1026</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4618,12 +4618,12 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>`mervärdskatt` (sv)</t>
+          <t>`glavå` (sv)</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1026</t>
         </is>
       </c>
     </row>
@@ -4640,12 +4640,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>`glavå` (sv)</t>
+          <t>`bargening` (en)</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
@@ -4657,7 +4657,7 @@
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>RV1026</t>
+          <t>RV1038</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -4667,17 +4667,17 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>`bargening` (en)</t>
+          <t>`obestånds` (sv)</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1026</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1038</t>
         </is>
       </c>
     </row>
@@ -4694,12 +4694,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>`obestånds` (sv)</t>
+          <t>`pratices` (en)</t>
         </is>
       </c>
       <c r="E158" s="2" t="inlineStr">
@@ -4726,7 +4726,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>`pratices` (en)</t>
+          <t>`securites` (en)</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
@@ -4738,7 +4738,7 @@
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>RV1038</t>
+          <t>RV1043</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4748,17 +4748,17 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>`securites` (en)</t>
+          <t>`förvaltningsrättliga` (sv)</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1038</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1043</t>
         </is>
       </c>
     </row>
@@ -4780,7 +4780,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>`förvaltningsrättliga` (sv)</t>
+          <t>`rättsäkerheten` (sv)</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr">
@@ -4792,7 +4792,7 @@
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>RV1043</t>
+          <t>RV1045</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4807,19 +4807,19 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>`rättsäkerheten` (sv)</t>
+          <t>`åtgärdscheman` (sv)</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1043</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1045</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>RV1045</t>
+          <t>RV1055</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4829,51 +4829,51 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>`åtgärdscheman` (sv)</t>
+          <t>`samt` — …aminationsformer  En kortare dugga per rättsområde (4x1 hp) samt samt en skriftlig inlämningsuppgift med avslutande seminarie (3,…</t>
         </is>
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1045</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1055</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>RV1055</t>
+          <t>ASK22L</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>RVA</t>
+          <t>SKA</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>`samt` — …aminationsformer  En kortare dugga per rättsområde (4x1 hp) samt samt en skriftlig inlämningsuppgift med avslutande seminarie (3,…</t>
+          <t>`formes` (en)</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1055</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK22L</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>ASK22L</t>
+          <t>ASK22M</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4888,19 +4888,19 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>`formes` (en)</t>
+          <t>`reviewscrutiny` (en)</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK22L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK22M</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>ASK22M</t>
+          <t>ASK289</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4915,46 +4915,46 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>`reviewscrutiny` (en)</t>
+          <t>`compative` (en)</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK22M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK289</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>ASK289</t>
+          <t>GSO2PL</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>SKA</t>
+          <t>SOA</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>`compative` (en)</t>
+          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ASK289</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSO2PL</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>GSO2PL</t>
+          <t>SO1027</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -4964,51 +4964,51 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>`credits` — …7.5 credits, Psychological Perspectives on Social Work 7.5 credits credits and Welfare Measures and User Perspective 15 credits…</t>
+          <t>`abilty` (en)</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSO2PL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SO1027</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>SO1027</t>
+          <t>ATR26B</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>SOA</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>`abilty` (en)</t>
+          <t>`hållbarbetsmål` (sv)</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SO1027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATR26B</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>ATR26B</t>
+          <t>ATR2BJ</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -5018,24 +5018,24 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>`hållbarbetsmål` (sv)</t>
+          <t>`leaisure` (en)</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATR26B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATR2BJ</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>ATR2BJ</t>
+          <t>GTR22D</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -5045,17 +5045,17 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>`leaisure` (en)</t>
+          <t>`samhållsvetenskap` (sv)</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ATR2BJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR22D</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>`samhållsvetenskap` (sv)</t>
+          <t>`värderigsförmåga` (sv)</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -5089,7 +5089,7 @@
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>GTR22D</t>
+          <t>GTR265</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -5104,12 +5104,12 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>`värderigsförmåga` (sv)</t>
+          <t>`fömåga` (sv)</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR22D</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR265</t>
         </is>
       </c>
     </row>
@@ -5126,12 +5126,12 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>`fömåga` (sv)</t>
+          <t>`afte` (en)</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
@@ -5143,7 +5143,7 @@
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>GTR265</t>
+          <t>GTR26E</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -5153,24 +5153,24 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>`afte` (en)</t>
+          <t>`erätter` (sv)</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR265</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR26E</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>GTR26E</t>
+          <t>GTR29Q</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -5185,12 +5185,12 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>`erätter` (sv)</t>
+          <t>`förhållningssät` (sv)</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR26E</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR29Q</t>
         </is>
       </c>
     </row>
@@ -5207,12 +5207,12 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>`förhållningssät` (sv)</t>
+          <t>`assignement` (en)</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>`assignement` (en)</t>
+          <t>`implmented` (en)</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
@@ -5251,7 +5251,7 @@
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>GTR29Q</t>
+          <t>GTR2DG</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -5261,17 +5261,17 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>`implmented` (en)</t>
+          <t>`the` — …earch. The course is organised into two parts. In part one, the The course introduces students to quantitative research. The co…</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR29Q</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR2DG</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5288,12 @@
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>`the` — …earch. The course is organised into two parts. In part one, the The course introduces students to quantitative research. The co…</t>
+          <t>`enkätsstudie` (sv)</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>GTR2DG</t>
+          <t>GTR2DP</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -5320,19 +5320,19 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>`enkätsstudie` (sv)</t>
+          <t>`värderingsfömåga` (sv)</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR2DG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR2DP</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>GTR2DP</t>
+          <t>TR1007</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -5342,24 +5342,24 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>`värderingsfömåga` (sv)</t>
+          <t>`recourses` (en)</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR2DP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1007</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>TR1007</t>
+          <t>TR1013</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -5369,17 +5369,17 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>`recourses` (en)</t>
+          <t>`använding` (sv)</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1013</t>
         </is>
       </c>
     </row>
@@ -5396,12 +5396,12 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>`använding` (sv)</t>
+          <t>`lerning` (en)</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
@@ -5413,7 +5413,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>TR1013</t>
+          <t>TR1018</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -5428,19 +5428,19 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>`lerning` (en)</t>
+          <t>`geodemographic` (en)</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1018</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>TR1018</t>
+          <t>TR1024</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -5450,17 +5450,17 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>`geodemographic` (en)</t>
+          <t>`fömåga` (sv)</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1024</t>
         </is>
       </c>
     </row>
@@ -5477,12 +5477,12 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>`fömåga` (sv)</t>
+          <t>`afte` (en)</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr">
@@ -5494,7 +5494,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>TR1024</t>
+          <t>TR1027</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5504,17 +5504,17 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>`afte` (en)</t>
+          <t>`fömåga` (sv)</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1027</t>
         </is>
       </c>
     </row>
@@ -5531,12 +5531,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>`fömåga` (sv)</t>
+          <t>`afte` (en)</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr">
@@ -5548,7 +5548,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>TR1027</t>
+          <t>TR1028</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5558,17 +5558,17 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>`afte` (en)</t>
+          <t>`förhållningssät` (sv)</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1027</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1028</t>
         </is>
       </c>
     </row>
@@ -5585,12 +5585,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>`förhållningssät` (sv)</t>
+          <t>`ansd` (en)</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr">
@@ -5602,7 +5602,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>TR1028</t>
+          <t>TR1030</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5612,24 +5612,24 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>`ansd` (en)</t>
+          <t>`tillvägagångsätt` (sv)</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1028</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1030</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>TR1030</t>
+          <t>TR1031</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5644,19 +5644,19 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>`tillvägagångsätt` (sv)</t>
+          <t>`kulturellafördomar` (sv)</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1030</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1031</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>TR1031</t>
+          <t>TR1034</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5671,12 +5671,12 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>`kulturellafördomar` (sv)</t>
+          <t>`förvärvda` (sv)</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1031</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1034</t>
         </is>
       </c>
     </row>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>`förvärvda` (sv)</t>
+          <t>`organisaton` (en)</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr">
@@ -5710,7 +5710,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>TR1034</t>
+          <t>TR2004</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5725,19 +5725,19 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>`organisaton` (en)</t>
+          <t>`stuides` (en)</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1034</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR2004</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>TR2004</t>
+          <t>TR3006</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5747,17 +5747,17 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>`stuides` (en)</t>
+          <t>`the` — …- Independently identify and analyze scientific problems in the the relevant field of knowledge and conduct and report on a pro…</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR2004</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR3006</t>
         </is>
       </c>
     </row>
@@ -5774,12 +5774,12 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Dubblerat ord</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>`the` — …- Independently identify and analyze scientific problems in the the relevant field of knowledge and conduct and report on a pro…</t>
+          <t>`ocskå` (sv)</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -5791,34 +5791,34 @@
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>TR3006</t>
+          <t>AS2002</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>TRU</t>
+          <t>UVX</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>`ocskå` (sv)</t>
+          <t>`takenup` (en)</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR3006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS2002</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>AS2002</t>
+          <t>AS3002</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5833,19 +5833,19 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>`takenup` (en)</t>
+          <t>`teh` (en)</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS2002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3002</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>AS3002</t>
+          <t>AS3009</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5855,24 +5855,24 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>`teh` (en)</t>
+          <t>`literära` (sv)</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3002</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3009</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>AS3009</t>
+          <t>AS3012</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5882,24 +5882,24 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>`literära` (sv)</t>
+          <t>`outlineof` (en)</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3009</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3012</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>AS3012</t>
+          <t>AS4003</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5909,49 +5909,22 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>`outlineof` (en)</t>
+          <t>`angrepssätt` (sv)</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS3012</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="2" t="inlineStr">
-        <is>
-          <t>AS4003</t>
-        </is>
-      </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>UVX</t>
-        </is>
-      </c>
-      <c r="C204" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D204" t="inlineStr">
-        <is>
-          <t>`angrepssätt` (sv)</t>
-        </is>
-      </c>
-      <c r="E204" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AS4003</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E204"/>
+  <autoFilter ref="A1:E203"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -6357,8 +6330,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E202" r:id="rId402"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A203" r:id="rId403"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E203" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A204" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E204" r:id="rId406"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis and course plan documents across multiple programs
- Modified various Excel files related to analysis for programs IHV, IKS, and ISLL, reflecting changes in grading, examination forms, and course references.
- Updated Markdown files for course plans, correcting quality notes and spelling errors, and adjusting the number of quality notes as necessary.
- Ensured consistency in naming and references across documents, including updates to links and descriptions for clarity.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1164,17 +1164,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>RV1001</t>
+          <t>GTR29Q</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RVA</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2007-01-10</t>
+          <t>2019-05-22</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
@@ -1185,29 +1185,29 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>`glavå` (sv)</t>
+          <t>`förhållningssät` (sv)</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR29Q</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>RV1026</t>
+          <t>TR1028</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>RVA</t>
+          <t>TRU</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2007-05-30</t>
+          <t>2015-12-07</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1218,487 +1218,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>`glavå` (sv)</t>
+          <t>`förhållningssät` (sv)</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=RV1026</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>GTR29Q</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>TRU</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>2019-05-22</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>`förhållningssät` (sv)</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GTR29Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>TR1028</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>TRU</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>2015-12-07</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>`förhållningssät` (sv)</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=TR1028</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>HAFSA</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>2014-11-20</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>`västafrika` (sv)</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=HAFSA</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>KAPSG</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>2023-01-30</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>`jörgensen` (sv)</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KAPSG</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>KFPPG</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>2025-01-15</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>`göran` (sv)</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KFPPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>KFTKG</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>2021-03-23</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>2023-07-05</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>`åsa` (sv)</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KFTKG</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>KMLJG</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>2020-10-20</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>2023-07-05</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>`påbyggbar` (sv)</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMLJG</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>KMPTG</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>2025-01-15</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>`thorbjörn` (sv)</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KMPTG</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>LVALA</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>`fändrik` (sv)</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>LVALA</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>`grundlärar` (sv)</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>LVALA</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>`umeå` (sv)</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>LVALA</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>2025-06-17</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>`ämneslärar` (sv)</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=LVALA</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>SPARG</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>2025-04-16</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>`enström` (sv)</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SPARG</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>SSHVG</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>2021-06-16</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>`möjliggörandet` (sv)</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=SSHVG</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G37"/>
+  <autoFilter ref="A1:G23"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -1744,34 +1274,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G36" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G37" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix spelling errors and update corrections in analysis files
- Added correction for "samtidafrågor" to "samtida frågor" in populate_analysfiler.py.
- Updated various Excel files in the vault-dalarna-university directory to correct spelling errors and ensure consistency across documents.
- Adjusted Markdown files to reflect corrected spellings and provide accurate information.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
@@ -590,7 +590,11 @@
           <t>`berätttarelement` (sv)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>berättarelement</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBQ2WK</t>

</xml_diff>

<commit_message>
Update course plans for ENA and FRA programs: corrected quality notes, fixed spelling errors, and updated metadata. Adjusted learning outcomes and course descriptions for clarity and consistency across multiple documents.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Stavfel och språkbruk.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$H$3</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +28,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -441,8 +434,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="70" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,99 +470,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Förslag</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
           <t>Länk</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>GBQ3FG</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>BPO</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2025-02-27</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>`excercises` (en)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>exercises</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBQ3FG</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>GPG2SC</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PGA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2021-12-03</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>`samhällorienterande` (sv)</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>samhällsorienterande</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GPG2SC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>